<commit_message>
导出问题 head down center
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/SkillGraph.xlsx
+++ b/Design/Excel/ET/Datas/Game/SkillGraph.xlsx
@@ -691,7 +691,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{"guid":"426755b7-c39a-4524-9cb5-960a31a19c10","nodeType":11,"position":{"x":587.3333740234375,"y":114.66667175292969},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"10","isPeriodic":true,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":1,"stackLimit":1,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[{"_name":"CD.BeRecBlood","_hashCode":-1099994396,"_shortName":"被动回血","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"cancelOnAbilityEnd":true,"buffId":0}</t>
+          <t>{"guid":"426755b7-c39a-4524-9cb5-960a31a19c10","nodeType":11,"position":{"x":587.3333740234375,"y":114.66667175292969},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"10","isPeriodic":true,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":1,"stackLimit":1,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[{"Name":"CD.BeRecBlood","HashCode":-1099994396,"ShortName":"被动回血","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"cancelOnAbilityEnd":true,"buffId":0}</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{"guid":"d5809887-df6e-4604-bd09-36cef191ce83","nodeType":0,"position":{"x":113.33334350585938,"y":158.66667175292969},"targetType":1,"skillId":2001,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[{"eventType":2,"customEventTag":"","PortId":1103}]}</t>
+          <t>{"guid":"d5809887-df6e-4604-bd09-36cef191ce83","nodeType":0,"position":{"x":113.33334350585938,"y":158.66667175292969},"targetType":1,"skillId":2001,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[{"eventType":2,"customEventTag":"","PortId":1103}]}</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{"guid":"7eefd9ae-c57e-439d-b1b6-e7f4e52f2f6f","nodeType":10,"position":{"x":370.66665649414063,"y":484.66665649414063},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.BeRecBlood","_hashCode":-1099994396,"_shortName":"被动回血","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"7eefd9ae-c57e-439d-b1b6-e7f4e52f2f6f","nodeType":10,"position":{"x":370.66665649414063,"y":484.66665649414063},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.BeRecBlood","HashCode":-1099994396,"ShortName":"被动回血","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{"guid":"a8c2d6c0-65f1-4bed-8a6a-70197e84bb56","nodeType":2,"position":{"x":933.3333740234375,"y":226.66667175292969},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"healSourceType":0,"healFixedValue":2.0,"healFormula":"","healMMCType":0,"healSetByCallerKey":"","healMMCCaptureAttribute":202,"healMMCAttributeSource":0,"healMMCCoefficient":1.0,"healMMCUseSnapshot":true,"healMultiplyByStackCount":false,"healCalculationType":0}</t>
+          <t>{"guid":"a8c2d6c0-65f1-4bed-8a6a-70197e84bb56","nodeType":2,"position":{"x":933.3333740234375,"y":226.66667175292969},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"healSourceType":0,"healFixedValue":2.0,"healFormula":"","healMMCType":0,"healSetByCallerKey":"","healMMCCaptureAttribute":202,"healMMCAttributeSource":0,"healMMCCoefficient":1.0,"healMMCUseSnapshot":true,"healMultiplyByStackCount":false,"healCalculationType":0}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"guid":"d086a8c9-8557-4a61-8fd2-64b3c1e543a3","nodeType":14,"position":{"x":1148.666748046875,"y":206.66667175292969},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"positionBindingName":"head","textType":1,"fixedText":"","contextDataKey":"Heal","textColor":{"r":0.040635824203491211,"g":1.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"d086a8c9-8557-4a61-8fd2-64b3c1e543a3","nodeType":14,"position":{"x":1148.666748046875,"y":206.66667175292969},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"positionBindingName":"head","textType":1,"fixedText":"","contextDataKey":"Heal","textColor":{"r":0.040635824203491211,"g":1.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G9"/>
@@ -793,7 +793,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2019.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2019.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1825.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.Blood","_hashCode":274000851,"_shortName":"Blood","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1825.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.Blood","HashCode":274000851,"ShortName":"Blood","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{"guid":"c353e286-8ef0-460a-b917-887f2aeb390a","nodeType":14,"position":{"x":383.33334350585938,"y":-1531.3333740234375},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"c353e286-8ef0-460a-b917-887f2aeb390a","nodeType":14,"position":{"x":383.33334350585938,"y":-1531.3333740234375},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1002,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.Blood","_hashCode":274000851,"_shortName":"Blood","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]},{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1002,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.Blood","HashCode":274000851,"ShortName":"Blood","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]},{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{"guid":"cb1df36f-5729-423e-9d1a-287db5a433f0","nodeType":11,"position":{"x":-160.66665649414063,"y":-1761.3333740234375},"targetType":0,"assetTags":{"_tags":[{"_name":"Buff.DeBuff.Dot","_hashCode":-637848644,"_shortName":"Dot","_ancestorHashCodes":[937056111,321157895],"_ancestorNames":["Buff","Buff.DeBuff"]}]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"10","isPeriodic":true,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":1,"stackLimit":3,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":1,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"buffId":0}</t>
+          <t>{"guid":"cb1df36f-5729-423e-9d1a-287db5a433f0","nodeType":11,"position":{"x":-160.66665649414063,"y":-1761.3333740234375},"targetType":0,"assetTags":{"Tags":[{"Name":"Buff.DeBuff.Dot","HashCode":-637848644,"ShortName":"Dot","AncestorHashCodes":[937056111,321157895],"AncestorNames":["Buff","Buff.DeBuff"]}]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"10","isPeriodic":true,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":1,"stackLimit":3,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":1,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"buffId":0}</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.66665649414063,"y":-1786.666748046875},"targetType":1,"searchShapeType":1,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":5.0,"searchSectorRadius":5.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"_tags":[{"_name":"unitType.monster","_hashCode":-2021655864,"_shortName":"monster","_ancestorHashCodes":[1600484460],"_ancestorNames":["unitType"]}]},"searchExcludeTags":{"_tags":[]}}</t>
+          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.66665649414063,"y":-1786.666748046875},"targetType":1,"searchShapeType":1,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":5.0,"searchSectorRadius":5.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"Tags":[{"Name":"unitType.monster","HashCode":-2021655864,"ShortName":"monster","AncestorHashCodes":[1600484460],"AncestorNames":["unitType"]}]},"searchExcludeTags":{"Tags":[]}}</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>{"guid":"f8947676-1084-4228-b991-1509cc7fe851","nodeType":1,"position":{"x":195.33334350585938,"y":-1761.3333740234375},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":20.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":true,"damageCalculationType":0,"enableHitKnockback":false,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
+          <t>{"guid":"f8947676-1084-4228-b991-1509cc7fe851","nodeType":1,"position":{"x":195.33334350585938,"y":-1761.3333740234375},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":20.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":true,"damageCalculationType":0,"enableHitKnockback":false,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50006,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_attack_02.prefab","particleBindingName":"down","particleOffset":{"x":5.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50006,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_attack_02.prefab","particleBindingName":"down","particleOffset":{"x":5.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
         </is>
       </c>
       <c r="G19"/>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1220.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.FireCircle","_hashCode":522143731,"_shortName":"FireCircle","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1220.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.FireCircle","HashCode":522143731,"ShortName":"FireCircle","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1195.3333740234375,"y":-2003.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":-100.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1195.3333740234375,"y":-2003.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":-100.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>{"guid":"eae41233-d297-46fe-a6c8-0b5c876fbb2a","nodeType":1,"position":{"x":-97.333328247070313,"y":-1810.0},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":true,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
+          <t>{"guid":"eae41233-d297-46fe-a6c8-0b5c876fbb2a","nodeType":1,"position":{"x":-97.333328247070313,"y":-1810.0},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":true,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-881.3333740234375,"y":-1854.666748046875},"targetType":1,"skillId":7001,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.FireCircle","_hashCode":522143731,"_shortName":"FireCircle","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"ongoingBlockedTags":{"_tags":[{"_name":"Buff.DeBuff.Stun","_hashCode":1791562953,"_shortName":"Stun","_ancestorHashCodes":[937056111,321157895],"_ancestorNames":["Buff","Buff.DeBuff"]}]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-881.3333740234375,"y":-1854.666748046875},"targetType":1,"skillId":7001,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.FireCircle","HashCode":522143731,"ShortName":"FireCircle","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"ongoingBlockedTags":{"Tags":[{"Name":"Buff.DeBuff.Stun","HashCode":1791562953,"ShortName":"Stun","AncestorHashCodes":[937056111,321157895],"AncestorNames":["Buff","Buff.DeBuff"]}]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>{"guid":"90bacd9f-d882-4bba-aaa8-41ed993ac3ff","nodeType":8,"position":{"x":-419.33331298828125,"y":-1840.0},"targetType":2,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":false,"offsetAngle":0.0,"curveHeight":0.0,"projectileEntityId":50001,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_gandian_buff.prefab","speed":3.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"_tags":[]},"collisionExcludeTags":{"_tags":[]},"isBouncing":true,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
+          <t>{"guid":"90bacd9f-d882-4bba-aaa8-41ed993ac3ff","nodeType":8,"position":{"x":-419.33331298828125,"y":-1840.0},"targetType":2,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":false,"offsetAngle":0.0,"curveHeight":0.0,"projectileEntityId":50001,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_gandian_buff.prefab","speed":3.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"Tags":[]},"collisionExcludeTags":{"Tags":[]},"isBouncing":true,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>{"guid":"2d7e41c4-8e90-4b61-879c-4b2e5b9486db","nodeType":14,"position":{"x":180.0,"y":-1810.0},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.16293229162693024,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"2d7e41c4-8e90-4b61-879c-4b2e5b9486db","nodeType":14,"position":{"x":180.0,"y":-1810.0},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.16293229162693024,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G27"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1220.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.FireCircle","_hashCode":522143731,"_shortName":"FireCircle","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"1","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1220.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.FireCircle","HashCode":522143731,"ShortName":"FireCircle","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"1","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1851.3333740234375},"targetType":1,"skillId":1010,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.FireCircle","_hashCode":522143731,"_shortName":"FireCircle","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1851.3333740234375},"targetType":1,"skillId":1010,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.FireCircle","HashCode":522143731,"ShortName":"FireCircle","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1195.3333740234375,"y":-2013.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":-100.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1195.3333740234375,"y":-2013.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":-100.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>{"guid":"eae41233-d297-46fe-a6c8-0b5c876fbb2a","nodeType":1,"position":{"x":45.333343505859375,"y":-1806.666748046875},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":true,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
+          <t>{"guid":"eae41233-d297-46fe-a6c8-0b5c876fbb2a","nodeType":1,"position":{"x":45.333343505859375,"y":-1806.666748046875},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":true,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>{"guid":"90bacd9f-d882-4bba-aaa8-41ed993ac3ff","nodeType":8,"position":{"x":-400.66665649414063,"y":-1836.666748046875},"targetType":2,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":false,"offsetAngle":0.0,"curveHeight":0.0,"projectileEntityId":50001,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_gandian_buff.prefab","speed":3.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"_tags":[]},"collisionExcludeTags":{"_tags":[]},"isBouncing":true,"bounceTargetMode":0,"maxBounceCount":2,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":50.0}</t>
+          <t>{"guid":"90bacd9f-d882-4bba-aaa8-41ed993ac3ff","nodeType":8,"position":{"x":-400.66665649414063,"y":-1836.666748046875},"targetType":2,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":false,"offsetAngle":0.0,"curveHeight":0.0,"projectileEntityId":50001,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_gandian_buff.prefab","speed":3.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"Tags":[]},"collisionExcludeTags":{"Tags":[]},"isBouncing":true,"bounceTargetMode":0,"maxBounceCount":2,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":50.0}</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>{"guid":"2d7e41c4-8e90-4b61-879c-4b2e5b9486db","nodeType":14,"position":{"x":408.66665649414063,"y":-1747.3333740234375},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":0.0,"g":0.323091983795166,"b":1.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"2d7e41c4-8e90-4b61-879c-4b2e5b9486db","nodeType":14,"position":{"x":408.66665649414063,"y":-1747.3333740234375},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":0.0,"g":0.323091983795166,"b":1.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G35"/>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.God","_hashCode":1317201809,"_shortName":"God","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.God","HashCode":1317201809,"ShortName":"God","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>{"guid":"091ecddb-f80b-4c00-aa06-f9bc718618d2","nodeType":22,"position":{"x":-93.333328247070313,"y":-1708.666748046875},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"0.5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"displaceType":1,"speed":10.0,"distance":3.0,"minDistance":0.5,"pointSource":0,"pointBindingName":""}</t>
+          <t>{"guid":"091ecddb-f80b-4c00-aa06-f9bc718618d2","nodeType":22,"position":{"x":-93.333328247070313,"y":-1708.666748046875},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"0.5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"displaceType":1,"speed":10.0,"distance":3.0,"minDistance":0.5,"pointSource":0,"pointBindingName":""}</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.0,"y":-1786.666748046875},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":4.0,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"_tags":[{"_name":"unitType.monster","_hashCode":-2021655864,"_shortName":"monster","_ancestorHashCodes":[1600484460],"_ancestorNames":["unitType"]}]},"searchExcludeTags":{"_tags":[]}}</t>
+          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.0,"y":-1786.666748046875},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":4.0,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"Tags":[{"Name":"unitType.monster","HashCode":-2021655864,"ShortName":"monster","AncestorHashCodes":[1600484460],"AncestorNames":["unitType"]}]},"searchExcludeTags":{"Tags":[]}}</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1005,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.RecBlood","_hashCode":1043024739,"_shortName":"RecBlood","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]},{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1005,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.RecBlood","HashCode":1043024739,"ShortName":"RecBlood","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]},{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50009,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_zhandounuhou_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50009,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_zhandounuhou_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
         </is>
       </c>
       <c r="G43"/>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-924.6666259765625,"y":-1886.666748046875},"targetType":1,"skillId":1007,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.RecBlood","_hashCode":1163914435,"_shortName":"回血","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-924.6666259765625,"y":-1886.666748046875},"targetType":1,"skillId":1007,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.RecBlood","HashCode":1163914435,"ShortName":"回血","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1156.0,"y":-1801.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.RecBlood","_hashCode":1163914435,"_shortName":"回血","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1156.0,"y":-1801.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.RecBlood","HashCode":1163914435,"ShortName":"回血","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"3","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>{"guid":"6d127270-5aeb-4542-9183-8d2d028d6786","nodeType":2,"position":{"x":-550.6666259765625,"y":-2050.0},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"healSourceType":0,"healFixedValue":10.0,"healFormula":"","healMMCType":0,"healSetByCallerKey":"","healMMCCaptureAttribute":1007,"healMMCAttributeSource":0,"healMMCCoefficient":1.0,"healMMCUseSnapshot":true,"healMultiplyByStackCount":false,"healCalculationType":0}</t>
+          <t>{"guid":"6d127270-5aeb-4542-9183-8d2d028d6786","nodeType":2,"position":{"x":-550.6666259765625,"y":-2050.0},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"healSourceType":0,"healFixedValue":10.0,"healFormula":"","healMMCType":0,"healSetByCallerKey":"","healMMCCaptureAttribute":1007,"healMMCAttributeSource":0,"healMMCCoefficient":1.0,"healMMCUseSnapshot":true,"healMultiplyByStackCount":false,"healCalculationType":0}</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>{"guid":"becb4d53-8a9e-4dc0-95a3-618d1e79ecc7","nodeType":14,"position":{"x":-303.33331298828125,"y":-1952.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":1,"fixedText":"","contextDataKey":"Heal","textColor":{"r":0.25257891416549683,"g":0.96226418018341064,"b":0.1180134117603302,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"becb4d53-8a9e-4dc0-95a3-618d1e79ecc7","nodeType":14,"position":{"x":-303.33331298828125,"y":-1952.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":1,"fixedText":"","contextDataKey":"Heal","textColor":{"r":0.25257891416549683,"g":0.96226418018341064,"b":0.1180134117603302,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>{"guid":"3cc340e3-1583-428e-ada4-c4e8539725d6","nodeType":3,"position":{"x":-1256.0,"y":-2008.0},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":100.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":1006,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false}</t>
+          <t>{"guid":"3cc340e3-1583-428e-ada4-c4e8539725d6","nodeType":3,"position":{"x":-1256.0,"y":-2008.0},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":100.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":1006,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false}</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":-303.33331298828125,"y":-2072.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50004,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_skill_zhanshi_huifunengliang.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":-303.33331298828125,"y":-2072.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50004,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_skill_zhanshi_huifunengliang.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
         </is>
       </c>
       <c r="G50"/>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.RuFood","_hashCode":-1045902856,"_shortName":"RuFood","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.RuFood","HashCode":-1045902856,"ShortName":"RuFood","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -1703,12 +1703,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1003,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.RuFood","_hashCode":-1045902856,"_shortName":"RuFood","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]},{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1003,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.RuFood","HashCode":-1045902856,"ShortName":"RuFood","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]},{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>{"outputNodeGuid":"cb1df36f-5729-423e-9d1a-287db5a433f0","outputPortId":3001,"inputNodeGuid":"93ec5a43-cc34-4e4a-acb3-39da2f2c3010","inputPortId":7001}</t>
+          <t>{"outputNodeGuid":"432ff1e3-b18d-476d-af80-d39ddc07402a","outputPortId":2000539,"inputNodeGuid":"f73ba91e-a76b-456c-b19c-a5176809d5f5","inputPortId":7001}</t>
         </is>
       </c>
       <c r="H55"/>
@@ -1723,12 +1723,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":676.6666259765625,"y":-1998.0},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50007,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_zhanshi_jcjt_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":676.6666259765625,"y":-1998.0},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50007,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_zhanshi_jcjt_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>{"outputNodeGuid":"432ff1e3-b18d-476d-af80-d39ddc07402a","outputPortId":2000539,"inputNodeGuid":"f73ba91e-a76b-456c-b19c-a5176809d5f5","inputPortId":7001}</t>
+          <t>{"outputNodeGuid":"432ff1e3-b18d-476d-af80-d39ddc07402a","outputPortId":2315086,"inputNodeGuid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","inputPortId":7001}</t>
         </is>
       </c>
       <c r="H56"/>
@@ -1739,16 +1739,16 @@
       <c r="C57"/>
       <c r="D57"/>
       <c r="E57">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>{"guid":"93ec5a43-cc34-4e4a-acb3-39da2f2c3010","nodeType":12,"position":{"x":387.33334350585938,"y":-1790.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":true,"positionSource":2,"particleEntityId":50005,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Xuanyun_01.prefab","particleBindingName":"head","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":true,"particleLoop":true}</t>
+          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.0,"y":-1786.666748046875},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":5.0,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"Tags":[{"Name":"unitType.monster","HashCode":-2021655864,"ShortName":"monster","AncestorHashCodes":[1600484460],"AncestorNames":["unitType"]}]},"searchExcludeTags":{"Tags":[]}}</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>{"outputNodeGuid":"432ff1e3-b18d-476d-af80-d39ddc07402a","outputPortId":2315086,"inputNodeGuid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","inputPortId":7001}</t>
+          <t>{"outputNodeGuid":"432ff1e3-b18d-476d-af80-d39ddc07402a","outputPortId":2287012,"inputNodeGuid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","inputPortId":7001}</t>
         </is>
       </c>
       <c r="H57"/>
@@ -1759,16 +1759,16 @@
       <c r="C58"/>
       <c r="D58"/>
       <c r="E58">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.0,"y":-1786.666748046875},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":5.0,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"_tags":[{"_name":"unitType.monster","_hashCode":-2021655864,"_shortName":"monster","_ancestorHashCodes":[1600484460],"_ancestorNames":["unitType"]}]},"searchExcludeTags":{"_tags":[]}}</t>
+          <t>{"guid":"cb1df36f-5729-423e-9d1a-287db5a433f0","nodeType":11,"position":{"x":18.66668701171875,"y":-1819.3333740234375},"targetType":0,"assetTags":{"Tags":[{"Name":"Buff.DeBuff.Stun","HashCode":1791562953,"ShortName":"Stun","AncestorHashCodes":[937056111,321157895],"AncestorNames":["Buff","Buff.DeBuff"]}]},"grantedTags":{"Tags":[{"Name":"Buff.DeBuff.Stun","HashCode":1791562953,"ShortName":"Stun","AncestorHashCodes":[937056111,321157895],"AncestorNames":["Buff","Buff.DeBuff"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"4","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":1,"stackLimit":1,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":1,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"buffId":0}</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>{"outputNodeGuid":"432ff1e3-b18d-476d-af80-d39ddc07402a","outputPortId":2287012,"inputNodeGuid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","inputPortId":7001}</t>
+          <t>{"outputNodeGuid":"cb1df36f-5729-423e-9d1a-287db5a433f0","outputPortId":3001,"inputNodeGuid":"93ec5a43-cc34-4e4a-acb3-39da2f2c3010","inputPortId":7001}</t>
         </is>
       </c>
       <c r="H58"/>
@@ -1779,11 +1779,11 @@
       <c r="C59"/>
       <c r="D59"/>
       <c r="E59">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>{"guid":"cb1df36f-5729-423e-9d1a-287db5a433f0","nodeType":11,"position":{"x":18.66668701171875,"y":-1787.3333740234375},"targetType":0,"assetTags":{"_tags":[{"_name":"Buff.DeBuff.Stun","_hashCode":1791562953,"_shortName":"Stun","_ancestorHashCodes":[937056111,321157895],"_ancestorNames":["Buff","Buff.DeBuff"]}]},"grantedTags":{"_tags":[{"_name":"Buff.DeBuff.Stun","_hashCode":1791562953,"_shortName":"Stun","_ancestorHashCodes":[937056111,321157895],"_ancestorNames":["Buff","Buff.DeBuff"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"4","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":1,"stackLimit":1,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":1,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"buffId":0}</t>
+          <t>{"guid":"93ec5a43-cc34-4e4a-acb3-39da2f2c3010","nodeType":12,"position":{"x":408.66665649414063,"y":-1790.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":true,"positionSource":2,"particleEntityId":50005,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Xuanyun_01.prefab","particleBindingName":"head","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":true,"particleLoop":true}</t>
         </is>
       </c>
       <c r="G59"/>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.SpeedUp","_hashCode":-605747253,"_shortName":"急速","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"10","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.SpeedUp","HashCode":-605747253,"ShortName":"急速","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"10","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1009,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.SpeedUp","_hashCode":-605747253,"_shortName":"急速","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1009,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.SpeedUp","HashCode":-605747253,"ShortName":"急速","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>{"guid":"632c75e2-152b-4376-8e9e-62c0e74f92d0","nodeType":11,"position":{"x":-502.66665649414063,"y":-1890.666748046875},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"7","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":300,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":2,"stackLimit":1,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"buffId":0}</t>
+          <t>{"guid":"632c75e2-152b-4376-8e9e-62c0e74f92d0","nodeType":11,"position":{"x":-502.66665649414063,"y":-1890.666748046875},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"7","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":300,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":2,"stackLimit":1,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"buffId":0}</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1130.6666259765625,"y":-2232.0},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.Sweep","_hashCode":-303359587,"_shortName":"Sweep","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"1","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1130.6666259765625,"y":-2232.0},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.Sweep","HashCode":-303359587,"ShortName":"Sweep","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"1","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1130.6666259765625,"y":-2479.333251953125},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":-10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1130.6666259765625,"y":-2479.333251953125},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":1003,"operation":0,"magnitudeSourceType":0,"fixedValue":-10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-843.3333740234375,"y":-2480.0},"targetType":1,"skillId":1001,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.Sweep","_hashCode":-303359587,"_shortName":"Sweep","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-843.3333740234375,"y":-2480.0},"targetType":1,"skillId":1001,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.Sweep","HashCode":-303359587,"ShortName":"Sweep","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>{"guid":"f8947676-1084-4228-b991-1509cc7fe851","nodeType":1,"position":{"x":974.666748046875,"y":-2340.66650390625},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":2,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":1006,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":true,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
+          <t>{"guid":"f8947676-1084-4228-b991-1509cc7fe851","nodeType":1,"position":{"x":974.666748046875,"y":-2340.66650390625},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":2,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":1006,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":true,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":731.3333740234375,"y":-2344.0},"targetType":1,"searchShapeType":1,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":5.0,"searchSectorRadius":5.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"_tags":[{"_name":"unitType.monster","_hashCode":-2021655864,"_shortName":"monster","_ancestorHashCodes":[1600484460],"_ancestorNames":["unitType"]}]},"searchExcludeTags":{"_tags":[]}}</t>
+          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":731.3333740234375,"y":-2344.0},"targetType":1,"searchShapeType":1,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":5.0,"searchSectorRadius":5.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"Tags":[{"Name":"unitType.monster","HashCode":-2021655864,"ShortName":"monster","AncestorHashCodes":[1600484460],"AncestorNames":["unitType"]}]},"searchExcludeTags":{"Tags":[]}}</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":731.3333740234375,"y":-2491.333251953125},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50006,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_attack_02.prefab","particleBindingName":"down","particleOffset":{"x":5.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":731.3333740234375,"y":-2491.333251953125},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50006,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_attack_02.prefab","particleBindingName":"down","particleOffset":{"x":5.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>{"guid":"c353e286-8ef0-460a-b917-887f2aeb390a","nodeType":14,"position":{"x":1213.3333740234375,"y":-2354.66650390625},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"c353e286-8ef0-460a-b917-887f2aeb390a","nodeType":14,"position":{"x":1213.3333740234375,"y":-2354.66650390625},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G74"/>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>{"guid":"f8947676-1084-4228-b991-1509cc7fe851","nodeType":1,"position":{"x":1452.666748046875,"y":-2239.333251953125},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":false,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
+          <t>{"guid":"f8947676-1084-4228-b991-1509cc7fe851","nodeType":1,"position":{"x":1452.666748046875,"y":-2239.333251953125},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":10.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":false,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1144.0,"y":-2405.333251953125},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1144.0,"y":-2405.333251953125},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1067.3333740234375,"y":-2188.66650390625},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.ThreeFire","_hashCode":960327319,"_shortName":"ThreeFire","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"1","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1067.3333740234375,"y":-2188.66650390625},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.ThreeFire","HashCode":960327319,"ShortName":"ThreeFire","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"1","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-746.6666259765625,"y":-2405.333251953125},"targetType":1,"skillId":1008,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.ThreeFire","_hashCode":960327319,"_shortName":"ThreeFire","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-746.6666259765625,"y":-2405.333251953125},"targetType":1,"skillId":1008,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.ThreeFire","HashCode":960327319,"ShortName":"ThreeFire","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>{"guid":"ce857360-de7e-4457-b348-9c124ce98879","nodeType":8,"position":{"x":1040.666748046875,"y":-2305.333251953125},"targetType":2,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":true,"offsetAngle":30.0,"curveHeight":0.0,"projectileEntityId":50002,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_huoyandan01.prefab","speed":10.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"_tags":[]},"collisionExcludeTags":{"_tags":[]},"isBouncing":false,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
+          <t>{"guid":"ce857360-de7e-4457-b348-9c124ce98879","nodeType":8,"position":{"x":1040.666748046875,"y":-2305.333251953125},"targetType":2,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":true,"offsetAngle":30.0,"curveHeight":0.0,"projectileEntityId":50002,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_huoyandan01.prefab","speed":10.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"Tags":[]},"collisionExcludeTags":{"Tags":[]},"isBouncing":false,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>{"guid":"9a695e91-e218-425e-82ed-1e157bf1b014","nodeType":8,"position":{"x":1022.666748046875,"y":-2131.333251953125},"targetType":2,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":true,"offsetAngle":0.0,"curveHeight":0.0,"projectileEntityId":50002,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_huoyandan01.prefab","speed":10.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"_tags":[]},"collisionExcludeTags":{"_tags":[]},"isBouncing":false,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
+          <t>{"guid":"9a695e91-e218-425e-82ed-1e157bf1b014","nodeType":8,"position":{"x":1022.666748046875,"y":-2131.333251953125},"targetType":2,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":true,"offsetAngle":0.0,"curveHeight":0.0,"projectileEntityId":50002,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_huoyandan01.prefab","speed":10.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"Tags":[]},"collisionExcludeTags":{"Tags":[]},"isBouncing":false,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>{"guid":"d897a922-5756-42cf-ac65-90a48c1e5a17","nodeType":8,"position":{"x":1022.666748046875,"y":-1951.3333740234375},"targetType":2,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":true,"offsetAngle":-30.0,"curveHeight":0.0,"projectileEntityId":50002,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_huoyandan01.prefab","speed":10.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"_tags":[]},"collisionExcludeTags":{"_tags":[]},"isBouncing":false,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
+          <t>{"guid":"d897a922-5756-42cf-ac65-90a48c1e5a17","nodeType":8,"position":{"x":1022.666748046875,"y":-1951.3333740234375},"targetType":2,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"launchPositionSource":0,"launchBindingName":"center","targetPositionSource":1,"targetBindingName":"center","projectileTargetType":0,"flyOver":true,"offsetAngle":-30.0,"curveHeight":0.0,"projectileEntityId":50002,"projectilePrefab":null,"projectilePrefabPath":"Assets/Res/Entity/Effect/ef_fashi_huoyandan01.prefab","speed":10.0,"maxDistance":10.0,"collisionRadius":0.5,"isPiercing":false,"maxPierceCount":1,"collisionTargetTags":{"Tags":[]},"collisionExcludeTags":{"Tags":[]},"isBouncing":false,"bounceTargetMode":0,"maxBounceCount":3,"bounceSearchRadius":10.0,"canBounceToSameTarget":false,"excludeSourceCamp":true,"bounceAngleOffset":0.0}</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>{"guid":"c353e286-8ef0-460a-b917-887f2aeb390a","nodeType":14,"position":{"x":1677.3333740234375,"y":-2239.333251953125},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"c353e286-8ef0-460a-b917-887f2aeb390a","nodeType":14,"position":{"x":1677.3333740234375,"y":-2239.333251953125},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>{"guid":"091ecddb-f80b-4c00-aa06-f9bc718618d2","nodeType":22,"position":{"x":-93.333328247070313,"y":-1708.666748046875},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"0.5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"displaceType":0,"speed":10.0,"distance":3.0,"minDistance":0.5,"pointSource":0,"pointBindingName":""}</t>
+          <t>{"guid":"091ecddb-f80b-4c00-aa06-f9bc718618d2","nodeType":22,"position":{"x":-93.333328247070313,"y":-1708.666748046875},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"0.5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"displaceType":0,"speed":10.0,"distance":3.0,"minDistance":0.5,"pointSource":0,"pointBindingName":""}</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.Wan","_hashCode":87403585,"_shortName":"Wan","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.Wan","HashCode":87403585,"ShortName":"Wan","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"5","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.0,"y":-1786.666748046875},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":4.0,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"_tags":[{"_name":"unitType.monster","_hashCode":-2021655864,"_shortName":"monster","_ancestorHashCodes":[1600484460],"_ancestorNames":["unitType"]}]},"searchExcludeTags":{"_tags":[]}}</t>
+          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":-452.0,"y":-1786.666748046875},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":4.0,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"Tags":[{"Name":"unitType.monster","HashCode":-2021655864,"ShortName":"monster","AncestorHashCodes":[1600484460],"AncestorNames":["unitType"]}]},"searchExcludeTags":{"Tags":[]}}</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1006,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.Wan","_hashCode":87403585,"_shortName":"Wan","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]},{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1006,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.Wan","HashCode":87403585,"ShortName":"Wan","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]},{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50010,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_zhentianpaoxiao_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":0,"particleEntityId":50010,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_Zhanshi_zhentianpaoxiao_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":false,"particleLoop":false}</t>
         </is>
       </c>
       <c r="G93"/>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"9d6f459d-b588-4b64-843b-1b71e8f299ae","nodeType":3,"position":{"x":-1186.6666259765625,"y":-2011.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[{"attrType":100,"operation":0,"magnitudeSourceType":0,"fixedValue":10.0,"formula":"","mmcType":0,"setByCallerKey":"","mmcCaptureAttribute":200,"mmcAttributeSource":0,"mmcCoefficient":1.0,"mmcUseSnapshot":true}],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>{"guid":"764289ea-065e-4f48-afc0-0f6963d18d57","nodeType":14,"position":{"x":492.00003051757813,"y":-1539.3333740234375},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
+          <t>{"guid":"764289ea-065e-4f48-afc0-0f6963d18d57","nodeType":14,"position":{"x":492.00003051757813,"y":-1539.3333740234375},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":false,"positionSource":2,"positionBindingName":"head","textType":0,"fixedText":"","contextDataKey":"DamageResult","textColor":{"r":1.0,"g":0.0,"b":0.0,"a":1.0},"criticalColor":{"r":1.0,"g":0.5,"b":0.0,"a":1.0},"missColor":{"r":0.5,"g":0.5,"b":0.5,"a":1.0},"fontSize":5.0,"criticalFontSize":60.0,"duration":1.5,"offset":{"x":0.0,"y":0.0},"moveDirection":{"x":0.0,"y":1.0}}</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>{"guid":"a32d1135-94db-4f81-95ba-9d5f105ef8d0","nodeType":1,"position":{"x":308.66665649414063,"y":-1720.0},"targetType":0,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":1.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":false,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
+          <t>{"guid":"a32d1135-94db-4f81-95ba-9d5f105ef8d0","nodeType":1,"position":{"x":308.66665649414063,"y":-1720.0},"targetType":0,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":0,"duration":"0","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true,"damageType":0,"damageSourceType":0,"damageFixedValue":1.0,"damageFormula":"","damageMMCType":0,"damageSetByCallerKey":"","damageMMCCaptureAttribute":200,"damageMMCAttributeSource":0,"damageMMCCoefficient":1.0,"damageMMCUseSnapshot":true,"damageMultiplyByStackCount":false,"damageCalculationType":0,"enableHitKnockback":false,"knockbackDistance":1.0,"knockbackSpeed":12.0}</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[{"_name":"CD.Wind","_hashCode":1982736573,"_shortName":"Wind","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]}]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":1,"duration":"15","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
+          <t>{"guid":"c28fb88d-51b1-47b2-be59-859e0ac638e3","nodeType":10,"position":{"x":-1186.6666259765625,"y":-1747.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[{"Name":"CD.Wind","HashCode":1982736573,"ShortName":"Wind","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]}]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":1,"duration":"15","isPeriodic":false,"period":"1","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":false,"cooldownType":0,"maxCharges":2,"chargeTime":"10"}</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>{"guid":"d8847c3e-459e-4589-a96b-37ebb5ec458b","nodeType":21,"position":{"x":-308.66665649414063,"y":-1769.3333740234375},"targetType":1,"assetTags":{"_tags":[]},"grantedTags":{"_tags":[]},"applicationRequiredTags":{"_tags":[]},"applicationImmunityTags":{"_tags":[]},"removeGameEffectsWithTags":{"_tags":[]},"durationType":2,"duration":"0","isPeriodic":true,"period":"0.3","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"_tags":[]},"cancelOnAbilityEnd":true}</t>
+          <t>{"guid":"d8847c3e-459e-4589-a96b-37ebb5ec458b","nodeType":21,"position":{"x":-308.66665649414063,"y":-1769.3333740234375},"targetType":1,"assetTags":{"Tags":[]},"grantedTags":{"Tags":[]},"applicationRequiredTags":{"Tags":[]},"applicationImmunityTags":{"Tags":[]},"removeGameEffectsWithTags":{"Tags":[]},"durationType":2,"duration":"0","isPeriodic":true,"period":"0.3","executeOnApplication":false,"attributeModifiers":[],"stackType":0,"stackLimit":0,"stackDurationRefreshPolicy":0,"stackPeriodResetPolicy":0,"stackExpirationPolicy":0,"stackOverflowPolicy":0,"ongoingRequiredTags":{"Tags":[]},"cancelOnAbilityEnd":true}</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":27.333343505859375,"y":-1769.3333740234375},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":2.5,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"_tags":[{"_name":"unitType.monster","_hashCode":-2021655864,"_shortName":"monster","_ancestorHashCodes":[1600484460],"_ancestorNames":["unitType"]}]},"searchExcludeTags":{"_tags":[]}}</t>
+          <t>{"guid":"e33ab94c-1496-4d6a-ba5e-1afd38bb0c30","nodeType":4,"position":{"x":27.333343505859375,"y":-1769.3333740234375},"targetType":1,"searchShapeType":0,"searchLineType":0,"positionSource":0,"positionBindingName":"center","searchCircleRadius":2.5,"searchSectorRadius":2.0,"searchSectorAngle":180.0,"searchLineDirectionOffsetAngle":0.0,"searchLineDirectionWidth":1.0,"searchLineDirectionLength":10.0,"lineStartPositionSource":0,"lineStartBindingName":"","lineEndPositionSource":1,"lineEndBindingName":"","searchLineBetweenWidth":1.0,"searchLineAbsoluteAngle":0.0,"searchLineAbsoluteWidth":1.0,"searchLineAbsoluteLength":10.0,"maxTargets":999,"searchTargetTags":{"Tags":[{"Name":"unitType.monster","HashCode":-2021655864,"ShortName":"monster","AncestorHashCodes":[1600484460],"AncestorNames":["unitType"]}]},"searchExcludeTags":{"Tags":[]}}</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1004,"assetTags":{"_tags":[]},"cancelAbilitiesWithTags":{"_tags":[]},"blockAbilitiesWithTags":{"_tags":[]},"activationOwnedTags":{"_tags":[{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"activationRequiredTags":{"_tags":[]},"activationBlockedTags":{"_tags":[{"_name":"CD.Wind","_hashCode":1982736573,"_shortName":"Wind","_ancestorHashCodes":[-1137859925],"_ancestorNames":["CD"]},{"_name":"Skill.Running","_hashCode":-51601538,"_shortName":"Running","_ancestorHashCodes":[1312877309],"_ancestorNames":["Skill"]}]},"ongoingBlockedTags":{"_tags":[]},"eventOutputPorts":[]}</t>
+          <t>{"guid":"356907e0-1488-4128-bfcc-7ff73cfc3330","nodeType":0,"position":{"x":-878.6666259765625,"y":-1853.3333740234375},"targetType":1,"skillId":1004,"assetTags":{"Tags":[]},"cancelAbilitiesWithTags":{"Tags":[]},"blockAbilitiesWithTags":{"Tags":[]},"activationOwnedTags":{"Tags":[{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"activationRequiredTags":{"Tags":[]},"activationBlockedTags":{"Tags":[{"Name":"CD.Wind","HashCode":1982736573,"ShortName":"Wind","AncestorHashCodes":[-1137859925],"AncestorNames":["CD"]},{"Name":"Skill.Running","HashCode":-51601538,"ShortName":"Running","AncestorHashCodes":[1312877309],"AncestorNames":["Skill"]}]},"ongoingBlockedTags":{"Tags":[]},"eventOutputPorts":[]}</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"_tags":[]},"immunityTags":{"_tags":[]},"destroyWithNode":true,"positionSource":0,"particleEntityId":50008,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_zhanshi_xfz_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":true,"particleLoop":true}</t>
+          <t>{"guid":"cde57fb8-b693-4da8-a4a8-fd61e56c5dcd","nodeType":12,"position":{"x":677.3333740234375,"y":-1998.666748046875},"targetType":1,"requiredTags":{"Tags":[]},"immunityTags":{"Tags":[]},"destroyWithNode":true,"positionSource":0,"particleEntityId":50008,"particlePrefab":null,"particlePrefabPath":"Assets/Res/Entity/Effect/ef_zhanshi_xfz_01.prefab","particleBindingName":"down","particleOffset":{"x":0.0,"y":0.0,"z":0.0},"particleScale":{"x":1.0,"y":1.0,"z":1.0},"attachToTarget":true,"particleLoop":true}</t>
         </is>
       </c>
       <c r="G103"/>

</xml_diff>